<commit_message>
add new (empty) sheet 'attachments'
</commit_message>
<xml_diff>
--- a/tricount_extractor/tests/data/expected_results/dinner_group_3.xlsx
+++ b/tricount_extractor/tests/data/expected_results/dinner_group_3.xlsx
@@ -10,7 +10,8 @@
     <sheet name="members" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="entries" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="allocations" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="balances" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="attachments" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="balances" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,16 +24,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -43,7 +41,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -51,21 +49,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -436,29 +425,29 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>member_id</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>member_uuid</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>member_name</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" t="n">
         <v>0</v>
       </c>
       <c r="B2" t="n">
@@ -481,7 +470,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" t="n">
         <v>1</v>
       </c>
       <c r="B3" t="n">
@@ -504,7 +493,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" t="n">
         <v>2</v>
       </c>
       <c r="B4" t="n">
@@ -541,55 +530,55 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>entry_id</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>amount</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>payer</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>is_reimbursement</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" t="n">
         <v>0</v>
       </c>
       <c r="B2" t="n">
         <v>3001</v>
       </c>
-      <c r="C2" s="2" t="n">
+      <c r="C2" s="1" t="n">
         <v>45689.79166666666</v>
       </c>
       <c r="D2" t="inlineStr">
@@ -634,55 +623,55 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>entry_id</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>payer</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>is_reimbursement</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>participant</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>share</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" t="n">
         <v>0</v>
       </c>
       <c r="B2" t="n">
         <v>3001</v>
       </c>
-      <c r="C2" s="2" t="n">
+      <c r="C2" s="1" t="n">
         <v>45689.79166666666</v>
       </c>
       <c r="D2" t="inlineStr">
@@ -713,13 +702,13 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" t="n">
         <v>1</v>
       </c>
       <c r="B3" t="n">
         <v>3001</v>
       </c>
-      <c r="C3" s="2" t="n">
+      <c r="C3" s="1" t="n">
         <v>45689.79166666666</v>
       </c>
       <c r="D3" t="inlineStr">
@@ -750,13 +739,13 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" t="n">
         <v>2</v>
       </c>
       <c r="B4" t="n">
         <v>3001</v>
       </c>
-      <c r="C4" s="2" t="n">
+      <c r="C4" s="1" t="n">
         <v>45689.79166666666</v>
       </c>
       <c r="D4" t="inlineStr">
@@ -797,23 +786,49 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="B1:C1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>entry_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>member</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>balance</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" t="n">
         <v>0</v>
       </c>
       <c r="B2" t="inlineStr">
@@ -826,7 +841,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" t="n">
         <v>1</v>
       </c>
       <c r="B3" t="inlineStr">
@@ -839,7 +854,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" t="n">
         <v>2</v>
       </c>
       <c r="B4" t="inlineStr">

</xml_diff>